<commit_message>
data: update depot type product list
</commit_message>
<xml_diff>
--- a/backend/stock/templates/Depo Tipi.xlsx
+++ b/backend/stock/templates/Depo Tipi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Metin\Desktop\Projeler\OMEGA\backend\stock\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E2599E-8478-4B08-8BB1-01C0B67D78DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0697F21F-C94D-4C2C-8E4D-CC8B582EF09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1500" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1520" uniqueCount="763">
   <si>
     <t>Ürün Kodu</t>
   </si>
@@ -2279,6 +2279,36 @@
   </si>
   <si>
     <t>806.264.18 Kahverengi Kilif</t>
+  </si>
+  <si>
+    <t>906.250.98 Bebek Battaniye</t>
+  </si>
+  <si>
+    <t>305.151.25 Bebek Battaniye Yesil</t>
+  </si>
+  <si>
+    <t>906.017.09 Duvar Saati</t>
+  </si>
+  <si>
+    <t>105.430.92 Duvar Saati Siyah</t>
+  </si>
+  <si>
+    <t>006.251.11 Bebek Havlu Tavsan</t>
+  </si>
+  <si>
+    <t>805.486.61 Organizer</t>
+  </si>
+  <si>
+    <t>304.444.68 Yatak Tepsisi</t>
+  </si>
+  <si>
+    <t>800.963.72 Abajur</t>
+  </si>
+  <si>
+    <t>104.610.10 Bel Yastigi</t>
+  </si>
+  <si>
+    <t>504.747.70 Monitor Stand</t>
   </si>
 </sst>
 </file>
@@ -2397,7 +2427,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tablo1" displayName="Tablo1" ref="A1:B750">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tablo1" displayName="Tablo1" ref="A1:B760">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Ürün Kodu"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Depo Tipi"/>
@@ -2607,7 +2637,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B750"/>
+  <dimension ref="A1:B760"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
@@ -8614,6 +8644,86 @@
         <v>3</v>
       </c>
     </row>
+    <row r="751" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A751" t="s">
+        <v>753</v>
+      </c>
+      <c r="B751" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="752" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A752" t="s">
+        <v>754</v>
+      </c>
+      <c r="B752" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="753" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A753" t="s">
+        <v>755</v>
+      </c>
+      <c r="B753" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="754" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A754" t="s">
+        <v>756</v>
+      </c>
+      <c r="B754" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="755" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A755" t="s">
+        <v>757</v>
+      </c>
+      <c r="B755" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="756" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A756" t="s">
+        <v>758</v>
+      </c>
+      <c r="B756" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="757" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A757" t="s">
+        <v>759</v>
+      </c>
+      <c r="B757" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="758" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A758" t="s">
+        <v>760</v>
+      </c>
+      <c r="B758" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="759" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A759" t="s">
+        <v>761</v>
+      </c>
+      <c r="B759" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="760" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A760" t="s">
+        <v>762</v>
+      </c>
+      <c r="B760" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>